<commit_message>
fix: align phase editing and point entry scope
</commit_message>
<xml_diff>
--- a/frontend/public/templates/优才计划积分批量导入模板_可打开版.xlsx
+++ b/frontend/public/templates/优才计划积分批量导入模板_可打开版.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="积分导入明细" sheetId="1" r:id="Ree8ee89317974ab8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="2" r:id="Rd3986c2321464306"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="选项字典" sheetId="3" r:id="R103422d07689422f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="积分导入明细" sheetId="1" r:id="Rc12d1e924b1a4ac7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="2" r:id="Rc8656ff2512e4c2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="选项字典" sheetId="3" r:id="Raef3d99e531548f9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -202,7 +202,7 @@
         <x:color rgb="FFB91C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE8E6"/>
         </x:patternFill>
       </x:fill>
@@ -213,7 +213,7 @@
         <x:color rgb="FF9C6500"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -289,9 +289,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -495,7 +495,7 @@
         <x:v>系统思维线上课程</x:v>
       </x:c>
       <x:c r="K2" s="13" t="str">
-        <x:v>3天内完成</x:v>
+        <x:v>发布后3天内完成</x:v>
       </x:c>
       <x:c r="L2" s="16" t="n">
         <x:v>15</x:v>
@@ -506,8 +506,8 @@
       <x:c r="N2" s="13" t="str">
         <x:v>学习平台导出</x:v>
       </x:c>
-      <x:c r="O2" s="13" t="str"/>
-      <x:c r="P2" s="13" t="str"/>
+      <x:c r="O2" s="13"/>
+      <x:c r="P2" s="13"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="13" t="str">
@@ -532,16 +532,16 @@
         <x:v>第二组</x:v>
       </x:c>
       <x:c r="H3" s="13" t="str">
-        <x:v>线上考试</x:v>
+        <x:v>学习输出</x:v>
       </x:c>
       <x:c r="I3" s="13" t="str">
-        <x:v>完成课程考试</x:v>
+        <x:v>完成个人学习感悟</x:v>
       </x:c>
       <x:c r="J3" s="13" t="str">
-        <x:v>系统思维考试</x:v>
+        <x:v>系统思维课后感悟</x:v>
       </x:c>
       <x:c r="K3" s="13" t="str">
-        <x:v>90分及以上</x:v>
+        <x:v>结合实际管理场景</x:v>
       </x:c>
       <x:c r="L3" s="16" t="n">
         <x:v>10</x:v>
@@ -550,12 +550,10 @@
         <x:v>46255</x:v>
       </x:c>
       <x:c r="N3" s="13" t="str">
-        <x:v>考试成绩导出</x:v>
-      </x:c>
-      <x:c r="O3" s="13" t="str"/>
-      <x:c r="P3" s="13" t="str">
-        <x:v>最终成绩95分</x:v>
-      </x:c>
+        <x:v>学员提交</x:v>
+      </x:c>
+      <x:c r="O3" s="13"/>
+      <x:c r="P3" s="13"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="13" t="str">
@@ -580,28 +578,28 @@
         <x:v>第一组</x:v>
       </x:c>
       <x:c r="H4" s="13" t="str">
-        <x:v>学习输出</x:v>
+        <x:v>问卷及测评反馈</x:v>
       </x:c>
       <x:c r="I4" s="13" t="str">
-        <x:v>课程学习输出</x:v>
+        <x:v>完成课程问卷</x:v>
       </x:c>
       <x:c r="J4" s="13" t="str">
-        <x:v>系统思维课后感悟</x:v>
+        <x:v>系统思维课程问卷</x:v>
       </x:c>
       <x:c r="K4" s="13" t="str">
-        <x:v>结合管理场景</x:v>
+        <x:v>规定时间内完整填写</x:v>
       </x:c>
       <x:c r="L4" s="16" t="n">
-        <x:v>10</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="M4" s="18" t="n">
         <x:v>46256</x:v>
       </x:c>
       <x:c r="N4" s="13" t="str">
-        <x:v>项目组评定</x:v>
-      </x:c>
-      <x:c r="O4" s="13" t="str"/>
-      <x:c r="P4" s="13" t="str"/>
+        <x:v>问卷记录</x:v>
+      </x:c>
+      <x:c r="O4" s="13"/>
+      <x:c r="P4" s="13"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="13" t="str">
@@ -629,7 +627,7 @@
         <x:v>课堂互动</x:v>
       </x:c>
       <x:c r="I5" s="13" t="str">
-        <x:v>扑克牌互动</x:v>
+        <x:v>有效案例分享</x:v>
       </x:c>
       <x:c r="J5" s="13" t="str">
         <x:v>课堂案例分享</x:v>
@@ -646,8 +644,8 @@
       <x:c r="N5" s="13" t="str">
         <x:v>课堂记录</x:v>
       </x:c>
-      <x:c r="O5" s="13" t="str"/>
-      <x:c r="P5" s="13" t="str"/>
+      <x:c r="O5" s="13"/>
+      <x:c r="P5" s="13"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="13" t="str">
@@ -672,28 +670,28 @@
         <x:v>第二组</x:v>
       </x:c>
       <x:c r="H6" s="13" t="str">
-        <x:v>实践任务</x:v>
+        <x:v>结营任务</x:v>
       </x:c>
       <x:c r="I6" s="13" t="str">
-        <x:v>阶段实践成果</x:v>
+        <x:v>完成个人结营任务</x:v>
       </x:c>
       <x:c r="J6" s="13" t="str">
-        <x:v>管理场景实践任务</x:v>
+        <x:v>个人结营成果</x:v>
       </x:c>
       <x:c r="K6" s="13" t="str">
-        <x:v>优秀</x:v>
+        <x:v>规定时间内提交</x:v>
       </x:c>
       <x:c r="L6" s="16" t="n">
-        <x:v>30</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="M6" s="18" t="n">
         <x:v>46266</x:v>
       </x:c>
       <x:c r="N6" s="13" t="str">
-        <x:v>项目组评定</x:v>
-      </x:c>
-      <x:c r="O6" s="13" t="str"/>
-      <x:c r="P6" s="13" t="str"/>
+        <x:v>学员提交</x:v>
+      </x:c>
+      <x:c r="O6" s="13"/>
+      <x:c r="P6" s="13"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="13"/>
@@ -18616,7 +18614,7 @@
       <x:formula>AND(A2&lt;&gt;"",COUNTIF($A$2:$A$1001,A2)&gt;1)</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:dataValidations count="4">
+  <x:dataValidations count="5">
     <x:dataValidation type="list" sqref="E2:E1001">
       <x:formula1>"优才计划,优才计划PLUS"</x:formula1>
     </x:dataValidation>
@@ -18629,10 +18627,13 @@
     <x:dataValidation type="list" sqref="N2:N1001">
       <x:formula1>"学习平台导出,考试成绩导出,签到记录,课堂记录,问卷记录,学员提交,小组长提报,讲师评定,项目组评定,特殊调整"</x:formula1>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="H2:H1000">
+      <x:formula1>"线上学习,学习输出,问卷及测评反馈,线下出勤,课堂互动,结营任务,小组长职责,特殊调整"</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b5aa363185b43a8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R41cdcc863d1d47e0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18833,7 +18834,7 @@
         <x:v>必填</x:v>
       </x:c>
       <x:c r="C17" s="13" t="str">
-        <x:v>填写具体课程、问卷、实践或活动名称</x:v>
+        <x:v>填写具体课程、问卷、结营任务或活动名称</x:v>
       </x:c>
       <x:c r="D17" s="13" t="str"/>
     </x:row>
@@ -18893,7 +18894,7 @@
         <x:v>按需填写</x:v>
       </x:c>
       <x:c r="C22" s="13" t="str">
-        <x:v>实践成果、项目贡献等可填写材料链接</x:v>
+        <x:v>可填写证明材料链接或特殊调整依据</x:v>
       </x:c>
       <x:c r="D22" s="13" t="str"/>
     </x:row>
@@ -19099,271 +19100,235 @@
       <x:c r="C9" s="12" t="str">
         <x:v>完成线上课程</x:v>
       </x:c>
-      <x:c r="D9" s="12" t="str"/>
+      <x:c r="D9" s="12"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="12" t="str">
         <x:v>积分类别</x:v>
       </x:c>
       <x:c r="B10" s="12" t="str">
-        <x:v>线上考试</x:v>
+        <x:v>学习输出</x:v>
       </x:c>
       <x:c r="C10" s="12" t="str">
-        <x:v>完成课程考试</x:v>
-      </x:c>
-      <x:c r="D10" s="12" t="str"/>
+        <x:v>完成个人学习感悟</x:v>
+      </x:c>
+      <x:c r="D10" s="12"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="12" t="str">
         <x:v>积分类别</x:v>
       </x:c>
       <x:c r="B11" s="12" t="str">
-        <x:v>学习输出</x:v>
+        <x:v>问卷及测评反馈</x:v>
       </x:c>
       <x:c r="C11" s="12" t="str">
-        <x:v>线上或线下课程后的学习感悟</x:v>
-      </x:c>
-      <x:c r="D11" s="12" t="str"/>
+        <x:v>课程、阶段、测评或结营反馈</x:v>
+      </x:c>
+      <x:c r="D11" s="12"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="12" t="str">
         <x:v>积分类别</x:v>
       </x:c>
       <x:c r="B12" s="12" t="str">
-        <x:v>问卷反馈</x:v>
+        <x:v>线下出勤</x:v>
       </x:c>
       <x:c r="C12" s="12" t="str">
-        <x:v>课程、培训或阶段问卷</x:v>
-      </x:c>
-      <x:c r="D12" s="12" t="str"/>
+        <x:v>线下集中培训签到</x:v>
+      </x:c>
+      <x:c r="D12" s="12"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="12" t="str">
         <x:v>积分类别</x:v>
       </x:c>
       <x:c r="B13" s="12" t="str">
-        <x:v>线下出勤</x:v>
+        <x:v>课堂互动</x:v>
       </x:c>
       <x:c r="C13" s="12" t="str">
-        <x:v>线下集中培训签到</x:v>
-      </x:c>
-      <x:c r="D13" s="12" t="str"/>
+        <x:v>回答问题或分享案例，按扑克牌计分</x:v>
+      </x:c>
+      <x:c r="D13" s="12"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="12" t="str">
         <x:v>积分类别</x:v>
       </x:c>
       <x:c r="B14" s="12" t="str">
-        <x:v>课堂互动</x:v>
+        <x:v>结营任务</x:v>
       </x:c>
       <x:c r="C14" s="12" t="str">
-        <x:v>扑克牌互动积分</x:v>
-      </x:c>
-      <x:c r="D14" s="12" t="str"/>
+        <x:v>完成个人结营任务</x:v>
+      </x:c>
+      <x:c r="D14" s="12"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="12" t="str">
         <x:v>积分类别</x:v>
       </x:c>
       <x:c r="B15" s="12" t="str">
-        <x:v>课堂任务</x:v>
+        <x:v>小组长职责</x:v>
       </x:c>
       <x:c r="C15" s="12" t="str">
-        <x:v>课堂个人或小组任务</x:v>
-      </x:c>
-      <x:c r="D15" s="12" t="str"/>
+        <x:v>阶段组织、提醒、推动及成果汇总</x:v>
+      </x:c>
+      <x:c r="D15" s="12"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="12" t="str">
         <x:v>积分类别</x:v>
       </x:c>
       <x:c r="B16" s="12" t="str">
-        <x:v>实践任务</x:v>
+        <x:v>特殊调整</x:v>
       </x:c>
       <x:c r="C16" s="12" t="str">
-        <x:v>阶段实践成果</x:v>
-      </x:c>
-      <x:c r="D16" s="12" t="str"/>
+        <x:v>补录、撤销和错误修正</x:v>
+      </x:c>
+      <x:c r="D16" s="12" t="str">
+        <x:v>必须填写调整原因</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="12" t="str">
-        <x:v>积分类别</x:v>
-      </x:c>
-      <x:c r="B17" s="12" t="str">
-        <x:v>成果转化</x:v>
-      </x:c>
-      <x:c r="C17" s="12" t="str">
-        <x:v>课程方法在工作中的应用</x:v>
-      </x:c>
-      <x:c r="D17" s="12" t="str"/>
+      <x:c r="A17" s="12"/>
+      <x:c r="B17" s="12"/>
+      <x:c r="C17" s="12"/>
+      <x:c r="D17" s="12"/>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="12" t="str">
-        <x:v>积分类别</x:v>
-      </x:c>
-      <x:c r="B18" s="12" t="str">
-        <x:v>团队共创</x:v>
-      </x:c>
-      <x:c r="C18" s="12" t="str">
-        <x:v>阶段小组任务</x:v>
-      </x:c>
-      <x:c r="D18" s="12" t="str"/>
+      <x:c r="A18" s="12"/>
+      <x:c r="B18" s="12"/>
+      <x:c r="C18" s="12"/>
+      <x:c r="D18" s="12"/>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="12" t="str">
-        <x:v>积分类别</x:v>
-      </x:c>
-      <x:c r="B19" s="12" t="str">
-        <x:v>团队贡献</x:v>
-      </x:c>
-      <x:c r="C19" s="12" t="str">
-        <x:v>成员承担关键职责</x:v>
-      </x:c>
-      <x:c r="D19" s="12" t="str"/>
+      <x:c r="A19" s="12"/>
+      <x:c r="B19" s="12"/>
+      <x:c r="C19" s="12"/>
+      <x:c r="D19" s="12"/>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="12" t="str">
-        <x:v>积分类别</x:v>
-      </x:c>
-      <x:c r="B20" s="12" t="str">
-        <x:v>小组长职责</x:v>
-      </x:c>
-      <x:c r="C20" s="12" t="str">
-        <x:v>小组组织及成果汇总</x:v>
-      </x:c>
-      <x:c r="D20" s="12" t="str"/>
+      <x:c r="A20" s="12"/>
+      <x:c r="B20" s="12"/>
+      <x:c r="C20" s="12"/>
+      <x:c r="D20" s="12"/>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="12" t="str">
-        <x:v>积分类别</x:v>
-      </x:c>
-      <x:c r="B21" s="12" t="str">
-        <x:v>项目贡献</x:v>
-      </x:c>
-      <x:c r="C21" s="12" t="str">
-        <x:v>分享、建议或运营协助</x:v>
-      </x:c>
-      <x:c r="D21" s="12" t="str"/>
+      <x:c r="A21" s="12"/>
+      <x:c r="B21" s="12"/>
+      <x:c r="C21" s="12"/>
+      <x:c r="D21" s="12"/>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="12" t="str">
-        <x:v>积分类别</x:v>
-      </x:c>
-      <x:c r="B22" s="12" t="str">
-        <x:v>特殊调整</x:v>
-      </x:c>
-      <x:c r="C22" s="12" t="str">
-        <x:v>补录、撤销和修正</x:v>
-      </x:c>
-      <x:c r="D22" s="12" t="str"/>
+      <x:c r="A22" s="12"/>
+      <x:c r="B22" s="12"/>
+      <x:c r="C22" s="12"/>
+      <x:c r="D22" s="12"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="12" t="str">
         <x:v>完成档位</x:v>
       </x:c>
       <x:c r="B23" s="12" t="str">
-        <x:v>3天内完成 / 按时完成 / 逾期完成</x:v>
+        <x:v>发布后3天内完成 / 规定时间内完成 / 逾期完成</x:v>
       </x:c>
       <x:c r="C23" s="12" t="str">
         <x:v>线上学习</x:v>
       </x:c>
-      <x:c r="D23" s="12" t="str"/>
+      <x:c r="D23" s="12"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="12" t="str">
         <x:v>完成档位</x:v>
       </x:c>
       <x:c r="B24" s="12" t="str">
-        <x:v>合格 / 80—89分 / 90分及以上</x:v>
+        <x:v>说明课程收获 / 结合实际管理场景 / 提出行动计划或改进方法</x:v>
       </x:c>
       <x:c r="C24" s="12" t="str">
-        <x:v>线上考试</x:v>
-      </x:c>
-      <x:c r="D24" s="12" t="str"/>
+        <x:v>学习输出</x:v>
+      </x:c>
+      <x:c r="D24" s="12"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="12" t="str">
         <x:v>完成档位</x:v>
       </x:c>
       <x:c r="B25" s="12" t="str">
-        <x:v>基础输出 / 结合管理场景 / 行动应用输出</x:v>
+        <x:v>规定时间内完整填写 / 未完成</x:v>
       </x:c>
       <x:c r="C25" s="12" t="str">
-        <x:v>学习输出</x:v>
-      </x:c>
-      <x:c r="D25" s="12" t="str"/>
+        <x:v>问卷及测评反馈</x:v>
+      </x:c>
+      <x:c r="D25" s="12"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="12" t="str">
         <x:v>完成档位</x:v>
       </x:c>
       <x:c r="B26" s="12" t="str">
-        <x:v>完整填写 / 有效建议</x:v>
+        <x:v>准时全程 / 迟到或早退10分钟内 / 超过10分钟或缺席</x:v>
       </x:c>
       <x:c r="C26" s="12" t="str">
-        <x:v>问卷反馈</x:v>
-      </x:c>
-      <x:c r="D26" s="12" t="str"/>
+        <x:v>线下出勤</x:v>
+      </x:c>
+      <x:c r="D26" s="12"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="12" t="str">
         <x:v>完成档位</x:v>
       </x:c>
       <x:c r="B27" s="12" t="str">
-        <x:v>全程参与 / 迟到或早退 / 完成补训</x:v>
+        <x:v>A / 2—10 / J / Q / K / 小王 / 大王</x:v>
       </x:c>
       <x:c r="C27" s="12" t="str">
-        <x:v>线下出勤</x:v>
-      </x:c>
-      <x:c r="D27" s="12" t="str"/>
+        <x:v>课堂互动</x:v>
+      </x:c>
+      <x:c r="D27" s="12" t="str">
+        <x:v>同一场每人最多2次</x:v>
+      </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="12" t="str">
         <x:v>完成档位</x:v>
       </x:c>
       <x:c r="B28" s="12" t="str">
-        <x:v>达标 / 优秀</x:v>
+        <x:v>按时提交 / 2个工作日内补交 / 超期或未提交</x:v>
       </x:c>
       <x:c r="C28" s="12" t="str">
-        <x:v>课堂任务、团队共创</x:v>
-      </x:c>
-      <x:c r="D28" s="12" t="str"/>
+        <x:v>结营任务</x:v>
+      </x:c>
+      <x:c r="D28" s="12"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="12" t="str">
         <x:v>完成档位</x:v>
       </x:c>
       <x:c r="B29" s="12" t="str">
-        <x:v>达标 / 良好 / 优秀</x:v>
+        <x:v>完成履职 / 未实际履职</x:v>
       </x:c>
       <x:c r="C29" s="12" t="str">
-        <x:v>实践任务</x:v>
-      </x:c>
-      <x:c r="D29" s="12" t="str"/>
+        <x:v>小组长职责</x:v>
+      </x:c>
+      <x:c r="D29" s="12"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="12" t="str">
         <x:v>完成档位</x:v>
       </x:c>
       <x:c r="B30" s="12" t="str">
-        <x:v>完成应用 / 形成案例 / 产生明显成效</x:v>
+        <x:v>按实际情况调整</x:v>
       </x:c>
       <x:c r="C30" s="12" t="str">
-        <x:v>成果转化</x:v>
-      </x:c>
-      <x:c r="D30" s="12" t="str"/>
+        <x:v>特殊调整</x:v>
+      </x:c>
+      <x:c r="D30" s="12" t="str">
+        <x:v>必须填写调整原因</x:v>
+      </x:c>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" s="12" t="str">
-        <x:v>完成档位</x:v>
-      </x:c>
-      <x:c r="B31" s="12" t="str">
-        <x:v>一般贡献 / 突出贡献</x:v>
-      </x:c>
-      <x:c r="C31" s="12" t="str">
-        <x:v>团队贡献、项目贡献</x:v>
-      </x:c>
-      <x:c r="D31" s="12" t="str"/>
+      <x:c r="A31" s="12"/>
+      <x:c r="B31" s="12"/>
+      <x:c r="C31" s="12"/>
+      <x:c r="D31" s="12"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="12" t="str">
@@ -19375,115 +19340,103 @@
       <x:c r="C32" s="12" t="str">
         <x:v>线上学习</x:v>
       </x:c>
-      <x:c r="D32" s="12" t="str"/>
+      <x:c r="D32" s="12"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="12" t="str">
         <x:v>数据来源</x:v>
       </x:c>
       <x:c r="B33" s="12" t="str">
-        <x:v>考试成绩导出</x:v>
+        <x:v>学员提交</x:v>
       </x:c>
       <x:c r="C33" s="12" t="str">
-        <x:v>线上考试</x:v>
-      </x:c>
-      <x:c r="D33" s="12" t="str"/>
+        <x:v>学习输出及结营任务</x:v>
+      </x:c>
+      <x:c r="D33" s="12"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="12" t="str">
         <x:v>数据来源</x:v>
       </x:c>
       <x:c r="B34" s="12" t="str">
-        <x:v>签到记录</x:v>
+        <x:v>问卷记录</x:v>
       </x:c>
       <x:c r="C34" s="12" t="str">
-        <x:v>线下出勤</x:v>
-      </x:c>
-      <x:c r="D34" s="12" t="str"/>
+        <x:v>问卷及测评反馈</x:v>
+      </x:c>
+      <x:c r="D34" s="12"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="12" t="str">
         <x:v>数据来源</x:v>
       </x:c>
       <x:c r="B35" s="12" t="str">
-        <x:v>课堂记录</x:v>
+        <x:v>签到记录</x:v>
       </x:c>
       <x:c r="C35" s="12" t="str">
-        <x:v>课堂互动及课堂任务</x:v>
-      </x:c>
-      <x:c r="D35" s="12" t="str"/>
+        <x:v>线下出勤</x:v>
+      </x:c>
+      <x:c r="D35" s="12"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="12" t="str">
         <x:v>数据来源</x:v>
       </x:c>
       <x:c r="B36" s="12" t="str">
-        <x:v>问卷记录</x:v>
+        <x:v>课堂记录</x:v>
       </x:c>
       <x:c r="C36" s="12" t="str">
-        <x:v>问卷反馈</x:v>
-      </x:c>
-      <x:c r="D36" s="12" t="str"/>
+        <x:v>课堂互动</x:v>
+      </x:c>
+      <x:c r="D36" s="12"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="12" t="str">
         <x:v>数据来源</x:v>
       </x:c>
       <x:c r="B37" s="12" t="str">
-        <x:v>学员提交</x:v>
+        <x:v>小组长提报</x:v>
       </x:c>
       <x:c r="C37" s="12" t="str">
-        <x:v>学习输出及实践成果</x:v>
-      </x:c>
-      <x:c r="D37" s="12" t="str"/>
+        <x:v>小组长职责</x:v>
+      </x:c>
+      <x:c r="D37" s="12"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="12" t="str">
         <x:v>数据来源</x:v>
       </x:c>
       <x:c r="B38" s="12" t="str">
-        <x:v>小组长提报</x:v>
+        <x:v>项目组评定</x:v>
       </x:c>
       <x:c r="C38" s="12" t="str">
-        <x:v>团队贡献</x:v>
-      </x:c>
-      <x:c r="D38" s="12" t="str"/>
+        <x:v>任务认定及综合评定</x:v>
+      </x:c>
+      <x:c r="D38" s="12"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="12" t="str">
         <x:v>数据来源</x:v>
       </x:c>
       <x:c r="B39" s="12" t="str">
-        <x:v>讲师评定</x:v>
+        <x:v>特殊调整</x:v>
       </x:c>
       <x:c r="C39" s="12" t="str">
-        <x:v>课堂或成果评定</x:v>
-      </x:c>
-      <x:c r="D39" s="12" t="str"/>
+        <x:v>补录或错误修正</x:v>
+      </x:c>
+      <x:c r="D39" s="12"/>
     </x:row>
     <x:row r="40">
-      <x:c r="A40" s="12" t="str">
-        <x:v>数据来源</x:v>
-      </x:c>
-      <x:c r="B40" s="12" t="str">
-        <x:v>项目组评定</x:v>
-      </x:c>
-      <x:c r="C40" s="12" t="str">
-        <x:v>项目贡献及综合评定</x:v>
-      </x:c>
-      <x:c r="D40" s="12" t="str"/>
+      <x:c r="A40" s="12"/>
+      <x:c r="B40" s="12"/>
+      <x:c r="C40" s="12"/>
+      <x:c r="D40" s="12"/>
     </x:row>
     <x:row r="41">
-      <x:c r="A41" s="12" t="str">
-        <x:v>数据来源</x:v>
-      </x:c>
-      <x:c r="B41" s="12" t="str">
-        <x:v>特殊调整</x:v>
-      </x:c>
-      <x:c r="C41" s="12" t="str">
-        <x:v>补录或错误修正</x:v>
-      </x:c>
-      <x:c r="D41" s="12" t="str"/>
+      <x:c r="A41" s="12"/>
+      <x:c r="B41" s="12"/>
+      <x:c r="C41" s="12"/>
+      <x:c r="D41" s="12"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>